<commit_message>
Auto sales drop update: 50100002-20260929.xlsx
</commit_message>
<xml_diff>
--- a/Reports/LY SEP.xlsx
+++ b/Reports/LY SEP.xlsx
@@ -16436,83 +16436,677 @@
       </c>
     </row>
     <row r="191" ht="18" customHeight="0">
-      <c s="5" t="inlineStr" r="A191">
+      <c s="3" r="A191">
+        <v>45928</v>
+      </c>
+      <c s="4" r="B191">
+        <v>45928</v>
+      </c>
+      <c s="5" t="inlineStr" r="C191">
+        <is>
+          <t xml:space="preserve">G-Sale</t>
+        </is>
+      </c>
+      <c s="6" r="D191">
+        <v>4304.000</v>
+      </c>
+      <c s="6" r="E191">
+        <v>1903.250</v>
+      </c>
+      <c s="6" r="F191">
+        <v>2097.000</v>
+      </c>
+      <c s="6" r="G191">
+        <v>531.000</v>
+      </c>
+      <c s="6" r="H191">
+        <v>1915.000</v>
+      </c>
+      <c s="6" r="I191">
+        <v>4552.000</v>
+      </c>
+      <c s="6" r="J191">
+        <v>2171.000</v>
+      </c>
+      <c s="6" r="K191">
+        <v>7250.000</v>
+      </c>
+      <c s="6" r="L191">
+        <v>1966.000</v>
+      </c>
+      <c s="6" r="M191">
+        <v>2600.000</v>
+      </c>
+      <c s="6" r="N191">
+        <v>1580.000</v>
+      </c>
+      <c s="6" r="O191">
+        <v>2915.000</v>
+      </c>
+      <c s="6" r="P191">
+        <v>1407.000</v>
+      </c>
+      <c s="6" r="Q191">
+        <v>2615.000</v>
+      </c>
+      <c s="6" r="R191">
+        <v>4686.700</v>
+      </c>
+      <c s="6" r="S191">
+        <v>537.000</v>
+      </c>
+      <c s="6" r="T191">
+        <v>5521.000</v>
+      </c>
+      <c s="6" r="U191">
+        <v>3431.000</v>
+      </c>
+      <c s="6" r="V191">
+        <v>2991.750</v>
+      </c>
+      <c s="6" r="W191">
+        <v>865.000</v>
+      </c>
+      <c s="7" r="X191">
+        <v>55838.700</v>
+      </c>
+    </row>
+    <row r="192" ht="18" customHeight="0">
+      <c s="8" t="str" r="A192"/>
+      <c s="5" t="inlineStr" r="B192">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C192">
+        <is>
+          <t xml:space="preserve">N-Sale</t>
+        </is>
+      </c>
+      <c s="9" r="D192">
+        <v>3742.680</v>
+      </c>
+      <c s="9" r="E192">
+        <v>1654.950</v>
+      </c>
+      <c s="9" r="F192">
+        <v>1823.450</v>
+      </c>
+      <c s="9" r="G192">
+        <v>461.730</v>
+      </c>
+      <c s="9" r="H192">
+        <v>1665.200</v>
+      </c>
+      <c s="9" r="I192">
+        <v>3958.280</v>
+      </c>
+      <c s="9" r="J192">
+        <v>1887.850</v>
+      </c>
+      <c s="9" r="K192">
+        <v>6304.348</v>
+      </c>
+      <c s="9" r="L192">
+        <v>1709.580</v>
+      </c>
+      <c s="9" r="M192">
+        <v>2260.870</v>
+      </c>
+      <c s="9" r="N192">
+        <v>1373.960</v>
+      </c>
+      <c s="9" r="O192">
+        <v>2534.790</v>
+      </c>
+      <c s="9" r="P192">
+        <v>1223.450</v>
+      </c>
+      <c s="9" r="Q192">
+        <v>2273.910</v>
+      </c>
+      <c s="9" r="R192">
+        <v>4075.290</v>
+      </c>
+      <c s="9" r="S192">
+        <v>466.960</v>
+      </c>
+      <c s="9" r="T192">
+        <v>4800.860</v>
+      </c>
+      <c s="9" r="U192">
+        <v>2983.450</v>
+      </c>
+      <c s="9" r="V192">
+        <v>2601.500</v>
+      </c>
+      <c s="9" r="W192">
+        <v>752.170</v>
+      </c>
+      <c s="10" r="X192">
+        <v>48555.278</v>
+      </c>
+    </row>
+    <row r="193" ht="18" customHeight="0">
+      <c s="11" t="inlineStr" r="A193">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B193">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C193">
+        <is>
+          <t xml:space="preserve">Quantity</t>
+        </is>
+      </c>
+      <c s="12" r="D193">
+        <v>204.00</v>
+      </c>
+      <c s="12" r="E193">
+        <v>115.00</v>
+      </c>
+      <c s="12" r="F193">
+        <v>24.00</v>
+      </c>
+      <c s="12" r="G193">
+        <v>9.00</v>
+      </c>
+      <c s="12" r="H193">
+        <v>13.00</v>
+      </c>
+      <c s="12" r="I193">
+        <v>22.00</v>
+      </c>
+      <c s="12" r="J193">
+        <v>11.00</v>
+      </c>
+      <c s="12" r="K193">
+        <v>371.00</v>
+      </c>
+      <c s="12" r="L193">
+        <v>99.00</v>
+      </c>
+      <c s="12" r="M193">
+        <v>159.00</v>
+      </c>
+      <c s="12" r="N193">
+        <v>137.00</v>
+      </c>
+      <c s="12" r="O193">
+        <v>140.00</v>
+      </c>
+      <c s="12" r="P193">
+        <v>15.00</v>
+      </c>
+      <c s="12" r="Q193">
+        <v>18.00</v>
+      </c>
+      <c s="12" r="R193">
+        <v>267.00</v>
+      </c>
+      <c s="12" r="S193">
+        <v>2.00</v>
+      </c>
+      <c s="12" r="T193">
+        <v>295.00</v>
+      </c>
+      <c s="12" r="U193">
+        <v>183.00</v>
+      </c>
+      <c s="12" r="V193">
+        <v>198.00</v>
+      </c>
+      <c s="12" r="W193">
+        <v>6.00</v>
+      </c>
+      <c s="10" r="X193">
+        <v>2288.00</v>
+      </c>
+    </row>
+    <row r="194" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A194">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B194">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C194">
+        <is>
+          <t xml:space="preserve">Transactions</t>
+        </is>
+      </c>
+      <c s="14" r="D194">
+        <v>72</v>
+      </c>
+      <c s="14" r="E194">
+        <v>34</v>
+      </c>
+      <c s="14" r="F194">
+        <v>9</v>
+      </c>
+      <c s="14" r="G194">
+        <v>2</v>
+      </c>
+      <c s="14" r="H194">
+        <v>9</v>
+      </c>
+      <c s="14" r="I194">
+        <v>13</v>
+      </c>
+      <c s="14" r="J194">
+        <v>8</v>
+      </c>
+      <c s="14" r="K194">
+        <v>81</v>
+      </c>
+      <c s="14" r="L194">
+        <v>37</v>
+      </c>
+      <c s="14" r="M194">
+        <v>43</v>
+      </c>
+      <c s="14" r="N194">
+        <v>48</v>
+      </c>
+      <c s="14" r="O194">
+        <v>72</v>
+      </c>
+      <c s="14" r="P194">
+        <v>7</v>
+      </c>
+      <c s="14" r="Q194">
+        <v>14</v>
+      </c>
+      <c s="14" r="R194">
+        <v>81</v>
+      </c>
+      <c s="14" r="S194">
+        <v>2</v>
+      </c>
+      <c s="14" r="T194">
+        <v>110</v>
+      </c>
+      <c s="14" r="U194">
+        <v>65</v>
+      </c>
+      <c s="14" r="V194">
+        <v>84</v>
+      </c>
+      <c s="14" r="W194">
+        <v>2</v>
+      </c>
+      <c s="15" r="X194">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="195" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A195">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B195">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C195">
+        <is>
+          <t xml:space="preserve">IPC/UPT</t>
+        </is>
+      </c>
+      <c s="9" r="D195">
+        <v>2.8333333333333333333333333333</v>
+      </c>
+      <c s="9" r="E195">
+        <v>5.75</v>
+      </c>
+      <c s="9" r="F195">
+        <v>2.6666666666666666666666666667</v>
+      </c>
+      <c s="9" r="G195">
+        <v>4.50</v>
+      </c>
+      <c s="9" r="H195">
+        <v>1.4444444444444444444444444444</v>
+      </c>
+      <c s="9" r="I195">
+        <v>1.6923076923076923076923076923</v>
+      </c>
+      <c s="9" r="J195">
+        <v>1.375</v>
+      </c>
+      <c s="9" r="K195">
+        <v>5.5373134328358208955223880597</v>
+      </c>
+      <c s="9" r="L195">
+        <v>2.6756756756756756756756756757</v>
+      </c>
+      <c s="9" r="M195">
+        <v>3.6976744186046511627906976744</v>
+      </c>
+      <c s="9" r="N195">
+        <v>2.8541666666666666666666666667</v>
+      </c>
+      <c s="9" r="O195">
+        <v>1.9444444444444444444444444444</v>
+      </c>
+      <c s="9" r="P195">
+        <v>2.1428571428571428571428571429</v>
+      </c>
+      <c s="9" r="Q195">
+        <v>1.2857142857142857142857142857</v>
+      </c>
+      <c s="9" r="R195">
+        <v>3.2962962962962962962962962963</v>
+      </c>
+      <c s="9" r="S195">
+        <v>1.00</v>
+      </c>
+      <c s="9" r="T195">
+        <v>2.6818181818181818181818181818</v>
+      </c>
+      <c s="9" r="U195">
+        <v>2.8153846153846153846153846154</v>
+      </c>
+      <c s="9" r="V195">
+        <v>2.3571428571428571428571428571</v>
+      </c>
+      <c s="9" r="W195">
+        <v>3.00</v>
+      </c>
+      <c s="10" r="X195">
+        <v>2.88524590163934</v>
+      </c>
+    </row>
+    <row r="196" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A196">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B196">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C196">
+        <is>
+          <t xml:space="preserve">ATV</t>
+        </is>
+      </c>
+      <c s="9" r="D196">
+        <v>51.981666666666666666666666667</v>
+      </c>
+      <c s="9" r="E196">
+        <v>48.675</v>
+      </c>
+      <c s="9" r="F196">
+        <v>202.60555555555555555555555556</v>
+      </c>
+      <c s="9" r="G196">
+        <v>230.865</v>
+      </c>
+      <c s="9" r="H196">
+        <v>185.02222222222222222222222222</v>
+      </c>
+      <c s="9" r="I196">
+        <v>304.48307692307692307692307692</v>
+      </c>
+      <c s="9" r="J196">
+        <v>235.98125</v>
+      </c>
+      <c s="9" r="K196">
+        <v>77.83145679012345679012345679</v>
+      </c>
+      <c s="9" r="L196">
+        <v>46.204864864864864864864864865</v>
+      </c>
+      <c s="9" r="M196">
+        <v>52.578372093023255813953488372</v>
+      </c>
+      <c s="9" r="N196">
+        <v>28.624166666666666666666666667</v>
+      </c>
+      <c s="9" r="O196">
+        <v>35.205416666666666666666666667</v>
+      </c>
+      <c s="9" r="P196">
+        <v>174.77857142857142857142857143</v>
+      </c>
+      <c s="9" r="Q196">
+        <v>162.42214285714285714285714286</v>
+      </c>
+      <c s="9" r="R196">
+        <v>50.312222222222222222222222222</v>
+      </c>
+      <c s="9" r="S196">
+        <v>233.480</v>
+      </c>
+      <c s="9" r="T196">
+        <v>43.644181818181818181818181818</v>
+      </c>
+      <c s="9" r="U196">
+        <v>45.899230769230769230769230769</v>
+      </c>
+      <c s="9" r="V196">
+        <v>30.970238095238095238095238095</v>
+      </c>
+      <c s="9" r="W196">
+        <v>376.085</v>
+      </c>
+      <c s="10" r="X196">
+        <v>61.2298587641866</v>
+      </c>
+    </row>
+    <row r="197" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="D197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="E197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="F197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="G197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="H197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="I197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="J197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="K197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="L197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="M197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="N197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="O197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="P197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="Q197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="R197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="S197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="T197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="U197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="V197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="W197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="X197">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="18" customHeight="0">
+      <c s="5" t="inlineStr" r="A198">
         <is>
           <t xml:space="preserve">Total</t>
         </is>
       </c>
-      <c s="1" t="inlineStr" r="B191">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="1" t="inlineStr" r="C191">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="17" r="D191">
-        <v>162935.717</v>
-      </c>
-      <c s="17" r="E191">
-        <v>74573.170</v>
-      </c>
-      <c s="17" r="F191">
-        <v>29617.967</v>
-      </c>
-      <c s="17" r="G191">
-        <v>34113.180</v>
-      </c>
-      <c s="17" r="H191">
-        <v>76141.999</v>
-      </c>
-      <c s="17" r="I191">
-        <v>82885.233</v>
-      </c>
-      <c s="17" r="J191">
-        <v>142299.400</v>
-      </c>
-      <c s="17" r="K191">
-        <v>326446.828</v>
-      </c>
-      <c s="17" r="L191">
-        <v>87058.033</v>
-      </c>
-      <c s="17" r="M191">
-        <v>166685.570</v>
-      </c>
-      <c s="17" r="N191">
-        <v>132695.750</v>
-      </c>
-      <c s="17" r="O191">
-        <v>114780.874</v>
-      </c>
-      <c s="17" r="P191">
-        <v>26747.560</v>
-      </c>
-      <c s="17" r="Q191">
-        <v>104417.020</v>
-      </c>
-      <c s="17" r="R191">
-        <v>139743.350</v>
-      </c>
-      <c s="17" r="S191">
-        <v>37726.300</v>
-      </c>
-      <c s="17" r="T191">
-        <v>256047.434</v>
-      </c>
-      <c s="17" r="U191">
-        <v>109897.085</v>
-      </c>
-      <c s="17" r="V191">
-        <v>102395.546</v>
-      </c>
-      <c s="17" r="W191">
-        <v>23146.374</v>
-      </c>
-      <c s="17" r="X191">
-        <v>2230354.390</v>
+      <c s="1" t="inlineStr" r="B198">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="1" t="inlineStr" r="C198">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="17" r="D198">
+        <v>166678.397</v>
+      </c>
+      <c s="17" r="E198">
+        <v>76228.120</v>
+      </c>
+      <c s="17" r="F198">
+        <v>31441.417</v>
+      </c>
+      <c s="17" r="G198">
+        <v>34574.910</v>
+      </c>
+      <c s="17" r="H198">
+        <v>77807.199</v>
+      </c>
+      <c s="17" r="I198">
+        <v>86843.513</v>
+      </c>
+      <c s="17" r="J198">
+        <v>144187.250</v>
+      </c>
+      <c s="17" r="K198">
+        <v>332751.176</v>
+      </c>
+      <c s="17" r="L198">
+        <v>88767.613</v>
+      </c>
+      <c s="17" r="M198">
+        <v>168946.440</v>
+      </c>
+      <c s="17" r="N198">
+        <v>134069.710</v>
+      </c>
+      <c s="17" r="O198">
+        <v>117315.664</v>
+      </c>
+      <c s="17" r="P198">
+        <v>27971.010</v>
+      </c>
+      <c s="17" r="Q198">
+        <v>106690.930</v>
+      </c>
+      <c s="17" r="R198">
+        <v>143818.640</v>
+      </c>
+      <c s="17" r="S198">
+        <v>38193.260</v>
+      </c>
+      <c s="17" r="T198">
+        <v>260848.294</v>
+      </c>
+      <c s="17" r="U198">
+        <v>112880.535</v>
+      </c>
+      <c s="17" r="V198">
+        <v>104997.046</v>
+      </c>
+      <c s="17" r="W198">
+        <v>23898.544</v>
+      </c>
+      <c s="17" r="X198">
+        <v>2278909.668</v>
       </c>
     </row>
   </sheetData>
@@ -16544,6 +17138,7 @@
     <mergeCell ref="A170:A171"/>
     <mergeCell ref="A177:A178"/>
     <mergeCell ref="A184:A185"/>
+    <mergeCell ref="A191:A192"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="1" footer="1"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Fix blank charts with resize event, add store-wise top/low 20 shoes filter, and implement opportunity-driven store IST logic
</commit_message>
<xml_diff>
--- a/Reports/LY SEP.xlsx
+++ b/Reports/LY SEP.xlsx
@@ -17624,83 +17624,677 @@
       </c>
     </row>
     <row r="205" ht="18" customHeight="0">
-      <c s="5" t="inlineStr" r="A205">
+      <c s="3" r="A205">
+        <v>45930</v>
+      </c>
+      <c s="4" r="B205">
+        <v>45930</v>
+      </c>
+      <c s="5" t="inlineStr" r="C205">
+        <is>
+          <t xml:space="preserve">G-Sale</t>
+        </is>
+      </c>
+      <c s="6" r="D205">
+        <v>5978.000</v>
+      </c>
+      <c s="6" r="E205">
+        <v>2664.400</v>
+      </c>
+      <c s="6" r="F205">
+        <v>1084.000</v>
+      </c>
+      <c s="6" r="G205">
+        <v>319.000</v>
+      </c>
+      <c s="6" r="H205">
+        <v>2076.000</v>
+      </c>
+      <c s="6" r="I205">
+        <v>3310.500</v>
+      </c>
+      <c s="6" r="J205">
+        <v>5230.500</v>
+      </c>
+      <c s="6" r="K205">
+        <v>7359.500</v>
+      </c>
+      <c s="6" r="L205">
+        <v>3622.600</v>
+      </c>
+      <c s="6" r="M205">
+        <v>5279.000</v>
+      </c>
+      <c s="6" r="N205">
+        <v>4031.000</v>
+      </c>
+      <c s="6" r="O205">
+        <v>3313.000</v>
+      </c>
+      <c s="6" r="P205">
+        <v>1320.000</v>
+      </c>
+      <c s="6" r="Q205">
+        <v>2041.000</v>
+      </c>
+      <c s="6" r="R205">
+        <v>3204.250</v>
+      </c>
+      <c s="6" r="S205">
+        <v>925.500</v>
+      </c>
+      <c s="6" r="T205">
+        <v>9630.000</v>
+      </c>
+      <c s="6" r="U205">
+        <v>4919.000</v>
+      </c>
+      <c s="6" r="V205">
+        <v>3749.000</v>
+      </c>
+      <c s="6" r="W205">
+        <v>1332.000</v>
+      </c>
+      <c s="7" r="X205">
+        <v>71388.250</v>
+      </c>
+    </row>
+    <row r="206" ht="18" customHeight="0">
+      <c s="8" t="str" r="A206"/>
+      <c s="5" t="inlineStr" r="B206">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C206">
+        <is>
+          <t xml:space="preserve">N-Sale</t>
+        </is>
+      </c>
+      <c s="9" r="D206">
+        <v>5198.261</v>
+      </c>
+      <c s="9" r="E206">
+        <v>2316.840</v>
+      </c>
+      <c s="9" r="F206">
+        <v>942.600</v>
+      </c>
+      <c s="9" r="G206">
+        <v>277.400</v>
+      </c>
+      <c s="9" r="H206">
+        <v>1805.220</v>
+      </c>
+      <c s="9" r="I206">
+        <v>2878.690</v>
+      </c>
+      <c s="9" r="J206">
+        <v>4548.260</v>
+      </c>
+      <c s="9" r="K206">
+        <v>6399.565</v>
+      </c>
+      <c s="9" r="L206">
+        <v>3150.110</v>
+      </c>
+      <c s="9" r="M206">
+        <v>4590.420</v>
+      </c>
+      <c s="9" r="N206">
+        <v>3505.220</v>
+      </c>
+      <c s="9" r="O206">
+        <v>2880.890</v>
+      </c>
+      <c s="9" r="P206">
+        <v>1147.790</v>
+      </c>
+      <c s="9" r="Q206">
+        <v>1774.780</v>
+      </c>
+      <c s="9" r="R206">
+        <v>2786.240</v>
+      </c>
+      <c s="9" r="S206">
+        <v>804.790</v>
+      </c>
+      <c s="9" r="T206">
+        <v>8373.880</v>
+      </c>
+      <c s="9" r="U206">
+        <v>4277.360</v>
+      </c>
+      <c s="9" r="V206">
+        <v>3259.980</v>
+      </c>
+      <c s="9" r="W206">
+        <v>1158.270</v>
+      </c>
+      <c s="10" r="X206">
+        <v>62076.566</v>
+      </c>
+    </row>
+    <row r="207" ht="18" customHeight="0">
+      <c s="11" t="inlineStr" r="A207">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B207">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C207">
+        <is>
+          <t xml:space="preserve">Quantity</t>
+        </is>
+      </c>
+      <c s="12" r="D207">
+        <v>294.00</v>
+      </c>
+      <c s="12" r="E207">
+        <v>168.00</v>
+      </c>
+      <c s="12" r="F207">
+        <v>7.00</v>
+      </c>
+      <c s="12" r="G207">
+        <v>2.00</v>
+      </c>
+      <c s="12" r="H207">
+        <v>13.00</v>
+      </c>
+      <c s="12" r="I207">
+        <v>17.00</v>
+      </c>
+      <c s="12" r="J207">
+        <v>30.00</v>
+      </c>
+      <c s="12" r="K207">
+        <v>347.00</v>
+      </c>
+      <c s="12" r="L207">
+        <v>193.00</v>
+      </c>
+      <c s="12" r="M207">
+        <v>251.00</v>
+      </c>
+      <c s="12" r="N207">
+        <v>240.00</v>
+      </c>
+      <c s="12" r="O207">
+        <v>213.00</v>
+      </c>
+      <c s="12" r="P207">
+        <v>9.00</v>
+      </c>
+      <c s="12" r="Q207">
+        <v>10.00</v>
+      </c>
+      <c s="12" r="R207">
+        <v>178.00</v>
+      </c>
+      <c s="12" r="S207">
+        <v>5.00</v>
+      </c>
+      <c s="12" r="T207">
+        <v>567.00</v>
+      </c>
+      <c s="12" r="U207">
+        <v>272.00</v>
+      </c>
+      <c s="12" r="V207">
+        <v>235.00</v>
+      </c>
+      <c s="12" r="W207">
+        <v>9.00</v>
+      </c>
+      <c s="10" r="X207">
+        <v>3060.00</v>
+      </c>
+    </row>
+    <row r="208" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A208">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B208">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C208">
+        <is>
+          <t xml:space="preserve">Transactions</t>
+        </is>
+      </c>
+      <c s="14" r="D208">
+        <v>96</v>
+      </c>
+      <c s="14" r="E208">
+        <v>41</v>
+      </c>
+      <c s="14" r="F208">
+        <v>6</v>
+      </c>
+      <c s="14" r="G208">
+        <v>3</v>
+      </c>
+      <c s="14" r="H208">
+        <v>9</v>
+      </c>
+      <c s="14" r="I208">
+        <v>14</v>
+      </c>
+      <c s="14" r="J208">
+        <v>19</v>
+      </c>
+      <c s="14" r="K208">
+        <v>104</v>
+      </c>
+      <c s="14" r="L208">
+        <v>60</v>
+      </c>
+      <c s="14" r="M208">
+        <v>76</v>
+      </c>
+      <c s="14" r="N208">
+        <v>86</v>
+      </c>
+      <c s="14" r="O208">
+        <v>75</v>
+      </c>
+      <c s="14" r="P208">
+        <v>4</v>
+      </c>
+      <c s="14" r="Q208">
+        <v>7</v>
+      </c>
+      <c s="14" r="R208">
+        <v>69</v>
+      </c>
+      <c s="14" r="S208">
+        <v>5</v>
+      </c>
+      <c s="14" r="T208">
+        <v>181</v>
+      </c>
+      <c s="14" r="U208">
+        <v>77</v>
+      </c>
+      <c s="14" r="V208">
+        <v>96</v>
+      </c>
+      <c s="14" r="W208">
+        <v>5</v>
+      </c>
+      <c s="15" r="X208">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="209" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A209">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B209">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C209">
+        <is>
+          <t xml:space="preserve">IPC/UPT</t>
+        </is>
+      </c>
+      <c s="9" r="D209">
+        <v>3.0947368421052631578947368421</v>
+      </c>
+      <c s="9" r="E209">
+        <v>5.4193548387096774193548387097</v>
+      </c>
+      <c s="9" r="F209">
+        <v>1.1666666666666666666666666667</v>
+      </c>
+      <c s="9" r="G209">
+        <v>0.6666666666666666666666666667</v>
+      </c>
+      <c s="9" r="H209">
+        <v>1.4444444444444444444444444444</v>
+      </c>
+      <c s="9" r="I209">
+        <v>1.2142857142857142857142857143</v>
+      </c>
+      <c s="9" r="J209">
+        <v>1.5789473684210526315789473684</v>
+      </c>
+      <c s="9" r="K209">
+        <v>3.3365384615384615384615384615</v>
+      </c>
+      <c s="9" r="L209">
+        <v>3.2166666666666666666666666667</v>
+      </c>
+      <c s="9" r="M209">
+        <v>3.3026315789473684210526315789</v>
+      </c>
+      <c s="9" r="N209">
+        <v>2.7906976744186046511627906977</v>
+      </c>
+      <c s="9" r="O209">
+        <v>2.84</v>
+      </c>
+      <c s="9" r="P209">
+        <v>2.25</v>
+      </c>
+      <c s="9" r="Q209">
+        <v>1.4285714285714285714285714286</v>
+      </c>
+      <c s="9" r="R209">
+        <v>2.579710144927536231884057971</v>
+      </c>
+      <c s="9" r="S209">
+        <v>1.00</v>
+      </c>
+      <c s="9" r="T209">
+        <v>3.1325966850828729281767955801</v>
+      </c>
+      <c s="9" r="U209">
+        <v>3.5324675324675324675324675325</v>
+      </c>
+      <c s="9" r="V209">
+        <v>2.4479166666666666666666666667</v>
+      </c>
+      <c s="9" r="W209">
+        <v>1.80</v>
+      </c>
+      <c s="10" r="X209">
+        <v>2.9622458857696</v>
+      </c>
+    </row>
+    <row r="210" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A210">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B210">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C210">
+        <is>
+          <t xml:space="preserve">ATV</t>
+        </is>
+      </c>
+      <c s="9" r="D210">
+        <v>54.148552083333333333333333333</v>
+      </c>
+      <c s="9" r="E210">
+        <v>56.508292682926829268292682927</v>
+      </c>
+      <c s="9" r="F210">
+        <v>157.100</v>
+      </c>
+      <c s="9" r="G210">
+        <v>92.46666666666666666666666667</v>
+      </c>
+      <c s="9" r="H210">
+        <v>200.580</v>
+      </c>
+      <c s="9" r="I210">
+        <v>205.62071428571428571428571429</v>
+      </c>
+      <c s="9" r="J210">
+        <v>239.38210526315789473684210526</v>
+      </c>
+      <c s="9" r="K210">
+        <v>61.534278846153846153846153846</v>
+      </c>
+      <c s="9" r="L210">
+        <v>52.501833333333333333333333333</v>
+      </c>
+      <c s="9" r="M210">
+        <v>60.400263157894736842105263158</v>
+      </c>
+      <c s="9" r="N210">
+        <v>40.758372093023255813953488372</v>
+      </c>
+      <c s="9" r="O210">
+        <v>38.411866666666666666666666667</v>
+      </c>
+      <c s="9" r="P210">
+        <v>286.9475</v>
+      </c>
+      <c s="9" r="Q210">
+        <v>253.540</v>
+      </c>
+      <c s="9" r="R210">
+        <v>40.380289855072463768115942029</v>
+      </c>
+      <c s="9" r="S210">
+        <v>160.958</v>
+      </c>
+      <c s="9" r="T210">
+        <v>46.264530386740331491712707182</v>
+      </c>
+      <c s="9" r="U210">
+        <v>55.55012987012987012987012987</v>
+      </c>
+      <c s="9" r="V210">
+        <v>33.958125</v>
+      </c>
+      <c s="9" r="W210">
+        <v>231.654</v>
+      </c>
+      <c s="10" r="X210">
+        <v>60.0934811229429</v>
+      </c>
+    </row>
+    <row r="211" ht="18" customHeight="0">
+      <c s="13" t="inlineStr" r="A211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="C211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="D211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="E211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="F211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="G211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="H211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="I211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="J211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="K211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="L211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="M211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="N211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="O211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="P211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="Q211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="R211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="S211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="T211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="U211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="V211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="W211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="13" t="inlineStr" r="X211">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="18" customHeight="0">
+      <c s="5" t="inlineStr" r="A212">
         <is>
           <t xml:space="preserve">Total</t>
         </is>
       </c>
-      <c s="1" t="inlineStr" r="B205">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="1" t="inlineStr" r="C205">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="17" r="D205">
-        <v>170725.571</v>
-      </c>
-      <c s="17" r="E205">
-        <v>78393.890</v>
-      </c>
-      <c s="17" r="F205">
-        <v>32340.537</v>
-      </c>
-      <c s="17" r="G205">
-        <v>37625.800</v>
-      </c>
-      <c s="17" r="H205">
-        <v>79981.059</v>
-      </c>
-      <c s="17" r="I205">
-        <v>88958.313</v>
-      </c>
-      <c s="17" r="J205">
-        <v>148708.430</v>
-      </c>
-      <c s="17" r="K205">
-        <v>338651.393</v>
-      </c>
-      <c s="17" r="L205">
-        <v>91064.113</v>
-      </c>
-      <c s="17" r="M205">
-        <v>171705.500</v>
-      </c>
-      <c s="17" r="N205">
-        <v>137353.180</v>
-      </c>
-      <c s="17" r="O205">
-        <v>120280.834</v>
-      </c>
-      <c s="17" r="P205">
-        <v>29476.210</v>
-      </c>
-      <c s="17" r="Q205">
-        <v>108725.710</v>
-      </c>
-      <c s="17" r="R205">
-        <v>147359.420</v>
-      </c>
-      <c s="17" r="S205">
-        <v>38375.000</v>
-      </c>
-      <c s="17" r="T205">
-        <v>267299.944</v>
-      </c>
-      <c s="17" r="U205">
-        <v>116902.885</v>
-      </c>
-      <c s="17" r="V205">
-        <v>107955.396</v>
-      </c>
-      <c s="17" r="W205">
-        <v>23942.024</v>
-      </c>
-      <c s="17" r="X205">
-        <v>2335825.209</v>
+      <c s="1" t="inlineStr" r="B212">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="1" t="inlineStr" r="C212">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="17" r="D212">
+        <v>175923.832</v>
+      </c>
+      <c s="17" r="E212">
+        <v>80710.730</v>
+      </c>
+      <c s="17" r="F212">
+        <v>33283.137</v>
+      </c>
+      <c s="17" r="G212">
+        <v>37903.200</v>
+      </c>
+      <c s="17" r="H212">
+        <v>81786.279</v>
+      </c>
+      <c s="17" r="I212">
+        <v>91837.003</v>
+      </c>
+      <c s="17" r="J212">
+        <v>153256.690</v>
+      </c>
+      <c s="17" r="K212">
+        <v>345050.958</v>
+      </c>
+      <c s="17" r="L212">
+        <v>94214.223</v>
+      </c>
+      <c s="17" r="M212">
+        <v>176295.920</v>
+      </c>
+      <c s="17" r="N212">
+        <v>140858.400</v>
+      </c>
+      <c s="17" r="O212">
+        <v>123161.724</v>
+      </c>
+      <c s="17" r="P212">
+        <v>30624.000</v>
+      </c>
+      <c s="17" r="Q212">
+        <v>110500.490</v>
+      </c>
+      <c s="17" r="R212">
+        <v>150145.660</v>
+      </c>
+      <c s="17" r="S212">
+        <v>39179.790</v>
+      </c>
+      <c s="17" r="T212">
+        <v>275673.824</v>
+      </c>
+      <c s="17" r="U212">
+        <v>121180.245</v>
+      </c>
+      <c s="17" r="V212">
+        <v>111215.376</v>
+      </c>
+      <c s="17" r="W212">
+        <v>25100.294</v>
+      </c>
+      <c s="17" r="X212">
+        <v>2397901.775</v>
       </c>
     </row>
   </sheetData>
@@ -17734,6 +18328,7 @@
     <mergeCell ref="A184:A185"/>
     <mergeCell ref="A191:A192"/>
     <mergeCell ref="A198:A199"/>
+    <mergeCell ref="A205:A206"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="1" footer="1"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>